<commit_message>
Mini-Boom en Cali v2: planeacion nocturna + rediseno visual homologado
- Movilidad reajustada al nuevo vuelo (ida 6pm, llega 8pm del 30): recomendado carro de agencia local que entrega coordinando el vuelo (cuadra con la llegada de noche); el mostrador de aeropuerto es mas barato pero cierra 10pm. Total recomendado Viajero + carro local ~$452k pp.

- Vehiculos: tabla de 7 puestos unificada a total de 3 dias con columna Por persona; Captiva Turbo (Farallones) corregida a ~$1.2M; locales (Fortuner, Montero, WayCarCali) + Kayak, con indicador de si cuadran con la llegada.

- Rediseno visual: sistema de tarjetas redondeadas con sombras suaves y paleta calida, luego calmado (colores unificados, sin figuras decorativas); emojis de criterio como ayuda visual; banderas en tarjeta.

- Estandar visual homologado a los 4 documentos (PDF con tarjetas/pildoras y recomendacion destacada; Excel y Markdown con emojis consistentes).

- Decision registrada en docs/bitacora-decisiones.md (D-004).
</commit_message>
<xml_diff>
--- a/output/Mini-Boom-en-Cali_Resultados.xlsx
+++ b/output/Mini-Boom-en-Cali_Resultados.xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movilidad" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntaje (metodología)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estadía (datos)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Económico" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amenidades en meta" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="El equilibrio" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casa entera" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vehículos (7 puestos)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntaje (metodología)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estadía (datos)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Económico" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amenidades en meta" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="El equilibrio" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casa entera" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,7 +171,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -572,21 +572,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Mini-Boom en Cali · Dossier de logística · transporte y estadía para siete</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
+          <t>Mini-Boom en Cali · Dossier de logística · transporte y estadía para siete (v2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>7 personas · 30 oct – 2 nov 2026 (viernes a lunes · 3 noches) · Salida 30 oct 7:00 am de Cartagena · regreso en vuelo 9:00 pm del 2 nov · Meta $300.000–$400.000 por persona (flex $480.000)</t>
+          <t>7 personas · 30 oct – 2 nov 2026 (viernes a lunes · 3 noches) · Ida 30 oct: sale 6:00 pm de Cartagena, llega 8:00 pm · regreso en vuelo 9:00 pm del 2 nov · Meta $300.000–$400.000 por persona (flex $480.000)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CUATRO LECTURAS (estadía + carro propio todo el viaje)</t>
+          <t>CUATRO LECTURAS (estadía + carro local con entrega)</t>
         </is>
       </c>
     </row>
@@ -642,10 +642,10 @@
         <v>89850</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>239850</v>
+        <v>289850</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
@@ -673,10 +673,10 @@
         <v>189750</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>339750</v>
+        <v>389750</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
@@ -704,10 +704,10 @@
         <v>252282</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>402282</v>
+        <v>452282</v>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
@@ -735,14 +735,14 @@
         <v>300000</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>450000</v>
+        <v>500000</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>EXCEDE</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -761,7 +761,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Viajero Hostel &amp; Salsa School + carro propio todo el viaje (recogido en el aeropuerto) ≈ $402.282 por persona</t>
+          <t>Viajero Hostel &amp; Salsa School + carro local con entrega coordinada ≈ $452.282 por persona</t>
         </is>
       </c>
     </row>
@@ -808,21 +808,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Movilidad — ¿en el aeropuerto o en la ciudad?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="58" customHeight="1">
+          <t>🌙 Movilidad — la llegada es de noche (v2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>En el aeropuerto, sin dudarlo. No hay que elegir entre barato y cómodo: hay agencias locales —más económicas que las marcas grandes— que o tienen oficina en el propio aeropuerto (Farallones) o llevan el carro hasta allá sin costo cuando el alquiler es de 3 días o más (WayCarCali). Se aterriza, se recoge el carro ahí mismo y se devuelve en el aeropuerto antes de volar. Ir hasta la ciudad a buscarlo solo agregaría un taxi y tiempo, sin ahorrar nada.</t>
+          <t>La llegada es a las 8 de la noche del 30, un viernes. El viaje entra en tres días de alquiler limpios (se recoge esa noche y se devuelve ~7 pm del 2, por debajo de las 72 horas). Para la hora, lo que mejor cuadra es una agencia local (Farallones, WayCarCali) que entrega el carro coordinando el vuelo. Los mostradores del aeropuerto (Alamo/Localiza) salen más baratos pero cierran ~10 pm, así que si se recoge ahí conviene reservar la recogida fuera de horario (24 h de aviso) por si el vuelo se retrasa. Y como red: los taxis oficiales del aeropuerto operan 24/7 (distintivo amarillo, tarifados, seguros).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Un detalle de horarios: el alquiler se cobra por días de 24 horas desde que se recoge, con una hora de gracia. Como se llega la mañana del 30 y se vuela a las 9 de la noche del 2, conservar el carro hasta esa noche cruza a un cuarto día de alquiler. Vale la pena: ese último tramo —entre dejar el hostal al mediodía y el vuelo de la noche— es justo cuando más sirve el carro, con las maletas ya encima. Si se devuelve de noche, conviene avisar a la agencia con un día de anticipación.</t>
+          <t>El alquiler se cuenta por días de 24 horas desde la recogida, con una hora de gracia; con la llegada de noche, los tres días cuadran hasta la tarde del 2. El matiz, corregido: el mostrador del aeropuerto sale un poco más barato pero tiene horario rígido (cierra ~10 pm); una agencia local cuesta algo más y, a cambio, entrega coordinando el vuelo — que es lo que de verdad cuadra con una llegada a las 8 pm.</t>
         </is>
       </c>
     </row>
@@ -856,20 +856,20 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Carro propio todo el viaje, recogido en el aeropuerto ★</t>
+          <t>Carro propio entregado por una agencia local (cuadra con la llegada de noche) ★</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Una van de 7 puestos de agencia local, recogida y devuelta en el mismo aeropuerto, manejándola ustedes, con la gasolina ya contada.</t>
+          <t>Una agencia local (Farallones, WayCarCali) entrega el carro coordinando el vuelo, sin pelear con el horario del mostrador; ~3 días con gasolina. P. ej. la Captiva Turbo (~$1.200.000 / 3 días).</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>La más cómoda: carro desde que aterrizan hasta que abordan, y libertad para salir de Cali cuando quieran (Pance, Calima).</t>
+          <t>La más libre y la que cuadra con la llegada de noche; cuesta un poco más que el mostrador.</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -881,20 +881,20 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Carro propio, pero solo tres días</t>
+          <t>Carro propio en el mostrador del aeropuerto (Kayak)</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Se devuelve al mediodía del último día para no pagar el cuarto día; esa última tarde se mueven en taxi, ya con las maletas.</t>
+          <t>Más barato (p. ej. Nissan X-Trail $1.033.028 / 3 días), pero el mostrador (Alamo/Localiza) cierra ~10 pm: con la llegada 8 pm va apretado, y si el vuelo se retrasa hay que reservar recogida fuera de horario (24 h de aviso).</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>140000</v>
+        <v>180000</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Ahorro pequeño; la última tarde quedan sin carro y cargando maletas.</t>
+          <t>El carro más barato, pero el horario del mostrador aprieta con la llegada de noche.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Taxis y apps dentro de la ciudad, más una van con conductor contratada solo para el día que salgan de Cali.</t>
+          <t>Taxi oficial de llegada (24/7), Uber/DiDi en la ciudad y una van con conductor contratada solo el día que salgan de Cali.</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -919,7 +919,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>La más barata y sin manejar ni parquear; a cambio, menos libertad para salir de improviso.</t>
+          <t>La más barata y sin manejar ni parquear; menos ideal si quieren varias salidas de la ciudad.</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -928,14 +928,11 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mostrador de marcas grandes en el aeropuerto (referencia, innecesario)</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="n">
-        <v>235000</v>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>La diferencia clave no es tanto el precio como el horario: el mostrador del aeropuerto es un poco más barato pero cierra ~10 pm; una agencia local cuesta algo más y entrega coordinando el vuelo, que es lo que cuadra con la llegada de las 8 pm. Los totales de 3 días de las locales se cierran por WhatsApp.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -982,26 +979,26 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Carro propio, pero solo tres días</t>
+          <t>Carro propio en el mostrador del aeropuerto (Kayak)</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>392282</v>
+        <v>432282</v>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>DENTRO</t>
+          <t>FLEX</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Carro propio todo el viaje, recogido en el aeropuerto</t>
+          <t>Carro propio entregado por una agencia local (cuadra con la llegada de noche)</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>402282</v>
+        <v>452282</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
@@ -1010,9 +1007,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
@@ -1025,6 +1023,278 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>🚙 Vehículos de 7 puestos — local (entrega) vs mostrador (Kayak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Todos los precios son por los 3 días, solo el alquiler (sin gasolina ni parqueo). Las tarifas locales 'desde' se calculan sobre la tarifa base/día × 3; en alquiler corto el total real suele ser mayor (la Captiva, confirmada, cuesta ~$1.200.000) — pidan el exacto por WhatsApp. Lo clave sigue siendo el horario: las locales entregan coordinando el vuelo; los mostradores cierran ~10 pm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Vehículo (7 puestos)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Agencia</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Tarifa (3 días)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Por persona</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>¿Cuadra con la llegada?</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Chevrolet Captiva Turbo</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Farallones (local)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>~$1.200.000</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>$171.429</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Sí — oficina en el aeropuerto y domicilio</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Toyota Fortuner</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Farallones (local)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>desde $1.140.000</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>$162.857</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Sí — entrega coordinando el vuelo</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Mitsubishi Montero Sport</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Farallones (local)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>desde $705.000</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>$100.714</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Sí — entrega coordinando el vuelo</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>7 puestos (varios modelos)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>WayCarCali (local)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>desde $360.000</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>$51.429</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Sí — domicilio gratis al aeropuerto (3+ días)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Nissan X-Trail</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Kayak · EconomyBookings</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>$1.033.028</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>$147.575</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Mostrador: cierra ~10 pm</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>SUV mediano híbrido</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Kayak · Alkilautos</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>$1.847.639</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>$263.948</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Mostrador: cierra ~10 pm</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1047,7 +1317,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cómo se compone el puntaje de estadía (0–100)</t>
+          <t>🎯 Cómo se compone el puntaje de estadía (0–100)</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1399,7 @@
       <c r="G5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="18" t="n">
         <v>77.59999999999999</v>
       </c>
       <c r="I5" s="15" t="n">
@@ -1160,7 +1430,7 @@
       <c r="G6" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="19" t="n">
         <v>75.8</v>
       </c>
       <c r="I6" s="11" t="n">
@@ -1191,7 +1461,7 @@
       <c r="G7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="20" t="n">
         <v>75.40000000000001</v>
       </c>
       <c r="I7" s="7" t="n">
@@ -1222,7 +1492,7 @@
       <c r="G8" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="19" t="n">
         <v>74.8</v>
       </c>
       <c r="I8" s="11" t="n">
@@ -1253,7 +1523,7 @@
       <c r="G9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="21" t="n">
+      <c r="H9" s="20" t="n">
         <v>72.8</v>
       </c>
       <c r="I9" s="7" t="n">
@@ -1284,7 +1554,7 @@
       <c r="G10" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="19" t="n">
         <v>71.2</v>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -1302,7 +1572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1324,7 +1594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Estadía — candidatos scrapeados (Hostelworld, fechas reales)</t>
+          <t>🏨 Estadía — candidatos scrapeados (Hostelworld, fechas reales)</t>
         </is>
       </c>
     </row>
@@ -1599,203 +1869,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Económico</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Máximo ahorro y el mejor rating del barrido (9.8). San Antonio, amenidades básicas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Detalle</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Por persona</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Grupo (×7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Estadía (3 noches)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>La Chanca Hostel</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>89850</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>628950</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Movilidad recomendada</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Carro propio todo el viaje, recogido en el aeropuerto</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>1050000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="inlineStr">
-        <is>
-          <t>Estado: DENTRO</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="n">
-        <v>239850</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>1678950</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Puntaje</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>74.8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Enlace</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>https://www.hostelworld.com/hostels/p/329092/la-chanca-hostel/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>Calificación huéspedes</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="n">
-        <v>9.800000000000001</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>Aire acondicionado</t>
-        </is>
-      </c>
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Piscina</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>Zona</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>San Antonio</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1819,14 +1892,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Amenidades en meta</t>
+          <t>Económico</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Piscina y aire acondicionado sin salir de los 400 mil. La alternativa prudente de presupuesto.</t>
+          <t>Máximo ahorro y el mejor rating del barrido (9.8). San Antonio, amenidades básicas.</t>
         </is>
       </c>
     </row>
@@ -1860,14 +1933,14 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Hostal Patio del Río</t>
+          <t>La Chanca Hostel</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>189750</v>
+        <v>89850</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1328250</v>
+        <v>628950</v>
       </c>
     </row>
     <row r="6">
@@ -1878,32 +1951,32 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Carro propio todo el viaje, recogido en el aeropuerto</t>
+          <t>Carro local (entrega)</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>1050000</v>
+        <v>1400000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Estado: DENTRO</t>
         </is>
       </c>
-      <c r="C7" s="23" t="n">
-        <v>339750</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>2378250</v>
+      <c r="C7" s="22" t="n">
+        <v>289850</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>2028950</v>
       </c>
     </row>
     <row r="9">
@@ -1913,7 +1986,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>72.8</v>
+        <v>74.8</v>
       </c>
     </row>
     <row r="10">
@@ -1924,65 +1997,65 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>https://www.hostelworld.com/hostels/p/323610/hostal-patio-del-rio/</t>
+          <t>https://www.hostelworld.com/hostels/p/329092/la-chanca-hostel/</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Calificación huéspedes</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
-        <v>9.6</v>
+      <c r="B12" s="23" t="n">
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Aire acondicionado</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Piscina</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Piscina</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>Oeste (Cali)</t>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
         </is>
       </c>
     </row>
@@ -2016,14 +2089,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>El equilibrio</t>
+          <t>Amenidades en meta</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Seguridad, piscina, aire, bar, rumba a pie y ambiente social. El puntaje más alto.</t>
+          <t>Piscina y aire acondicionado sin salir de los 400 mil. La alternativa prudente de presupuesto.</t>
         </is>
       </c>
     </row>
@@ -2057,14 +2130,14 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Viajero Hostel &amp; Salsa School</t>
+          <t>Hostal Patio del Río</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>252282</v>
+        <v>189750</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1765974</v>
+        <v>1328250</v>
       </c>
     </row>
     <row r="6">
@@ -2075,32 +2148,32 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Carro propio todo el viaje, recogido en el aeropuerto</t>
+          <t>Carro local (entrega)</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>1050000</v>
+        <v>1400000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>Estado: FLEX</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>402282</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>2815974</v>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Estado: DENTRO</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>389750</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>2728250</v>
       </c>
     </row>
     <row r="9">
@@ -2110,7 +2183,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>72.8</v>
       </c>
     </row>
     <row r="10">
@@ -2121,65 +2194,65 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>https://www.hostelworld.com/hostels/p/73676/viajero-cali-hostel-and-salsa-school/</t>
+          <t>https://www.hostelworld.com/hostels/p/323610/hostal-patio-del-rio/</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Calificación huéspedes</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="23" t="n">
         <v>9.6</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Aire acondicionado</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Piscina</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Cocina</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>San Antonio</t>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Oeste (Cali)</t>
         </is>
       </c>
     </row>
@@ -2213,14 +2286,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Casa entera</t>
+          <t>El equilibrio</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Máxima privacidad y comodidad (piscina, aire, cocina). Dentro del flex.</t>
+          <t>Seguridad, piscina, aire, bar, rumba a pie y ambiente social. El puntaje más alto.</t>
         </is>
       </c>
     </row>
@@ -2254,6 +2327,203 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
+          <t>Viajero Hostel &amp; Salsa School</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>252282</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1765974</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Movilidad recomendada</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Carro local (entrega)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>1400000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Estado: FLEX</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>452282</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>3165974</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Puntaje</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>77.59999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Enlace</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.hostelworld.com/hostels/p/73676/viajero-cali-hostel-and-salsa-school/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Calificación huéspedes</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Aire acondicionado</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Piscina</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Casa entera</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Máxima privacidad y comodidad (piscina, aire, cocina). Dentro del flex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Por persona</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Grupo (×7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Estadía (3 noches)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
           <t>Casa/Apto entero (Airbnb)</t>
         </is>
       </c>
@@ -2272,32 +2542,32 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Carro propio todo el viaje, recogido en el aeropuerto</t>
+          <t>Carro local (entrega)</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>1050000</v>
+        <v>1400000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
-        <is>
-          <t>Estado: FLEX</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="n">
-        <v>450000</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>3150000</v>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Estado: EXCEDE</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>3500000</v>
       </c>
     </row>
     <row r="9">
@@ -2323,60 +2593,60 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Calificación huéspedes</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Aire acondicionado</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Piscina</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Cocina</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>San Antonio (Oeste)</t>
         </is>

</xml_diff>

<commit_message>
Añade subsección Airbnb (casas/aptos enteros) con datos reales + dimensión de baños
- Scrapers nuevos: explora_airbnb.py (listados, alojamiento entero, zonas seguras)
  y explora_fichas_airbnb.py (capacidad, habitaciones, camas y baños por ficha).
  Barrido real con Playwright en el devcontainer, fechas 30 oct-2 nov, 7 personas.
- Dimensión de baños como informativa (columna '¿Baño compartido?'), sin tocar
  pesos ni filtros: el puntaje y el ranking de hostales quedan intactos.
- Subsección Airbnb en los 4 entregables (informe, Excel, PDF, presentación) con
  las mejores casas/aptos enteros y dos contraejemplos (por qué se miran baños y camas).
- Hallazgo: casa entera real desde ~$77k-90k pp/3n (muy por debajo del estimado
  viejo de $300k); la lectura 'Casa entera' pasa a $278.571 pp (DENTRO) con el precio real.
- Documenta D-005 en la bitácora y AIRBNB_ENTEROS en el diccionario de datos.
</commit_message>
<xml_diff>
--- a/output/Mini-Boom-en-Cali_Resultados.xlsx
+++ b/output/Mini-Boom-en-Cali_Resultados.xlsx
@@ -12,10 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vehículos (7 puestos)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntaje (metodología)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estadía (datos)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Económico" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amenidades en meta" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="El equilibrio" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casa entera" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Airbnb (enteros)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Económico" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amenidades en meta" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="El equilibrio" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casa entera" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -728,21 +729,21 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Casa/Apto entero (Airbnb)</t>
+          <t>Casa de 4 Habitaciones – Terraza y Aire/C</t>
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>300000</v>
+        <v>78571</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>200000</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>500000</v>
+        <v>278571</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>EXCEDE</t>
+          <t>DENTRO</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -784,6 +785,205 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId4"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Casa entera</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Baños del grupo, cocina y privacidad total. Precio real del barrido de Airbnb (ver subsección).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Por persona</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Grupo (×7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Estadía (3 noches)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Casa de 4 Habitaciones – Terraza y Aire/C</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>78571</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>549997</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Movilidad recomendada</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Carro local (entrega)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>1400000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Estado: DENTRO</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>278571</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>1949997</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Puntaje</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>71.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Enlace</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.com/s/San-Antonio--Cali--Valle-del-Cauca/homes?checkin=2026-10-30&amp;checkout=2026-11-02&amp;adults=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Calificación huéspedes</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Aire acondicionado</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Piscina</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>San Antonio (Oeste)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1578,7 +1778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1587,8 +1787,9 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1631,10 +1832,15 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
+          <t>¿Baño compartido?</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
           <t>Estadía por persona (3n)</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Ver</t>
         </is>
@@ -1667,10 +1873,15 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Depende*</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n">
         <v>252282</v>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -1703,10 +1914,15 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Depende*</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="n">
         <v>150000</v>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -1739,10 +1955,15 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Depende*</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n">
         <v>150000</v>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -1775,10 +1996,15 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Depende*</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="n">
         <v>89850</v>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -1811,10 +2037,15 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Depende*</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n">
         <v>189750</v>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -1849,26 +2080,39 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
       </c>
     </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>* El baño en hostal depende de la habitación (confirmar baño privado al reservar). En casa/apto entero NINGÚN baño se comparte — ver la hoja «Airbnb (enteros)». Dimensión informativa: no entra al puntaje.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A11:I11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1880,192 +2124,270 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Económico</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
+          <t>🛏️ Airbnb — casas y aptos enteros (baños del grupo, fechas reales)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Máximo ahorro y el mejor rating del barrido (9.8). San Antonio, amenidades básicas.</t>
+          <t>Barrido real con Playwright (alojamiento entero, 7 personas). Ningún baño se comparte con extraños. La casa entera había entrado al puntaje con un estimado de $300.000 pp; el barrido real la dejó desde ~$78.571 pp.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Casa / apto entero</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Detalle</t>
+          <t>Zona</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Por persona</t>
+          <t>Cabe</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Grupo (×7)</t>
+          <t>Camas</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Baños</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Aire</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Piscina</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Por persona (3n)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Ver</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Estadía (3 noches)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>La Chanca Hostel</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>89850</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>628950</v>
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Casa de 4 Habitaciones – Terraza y Aire/C ★</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Sí (anuncio)</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="n">
+        <v>78571</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Movilidad recomendada</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Carro local (entrega)</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>1400000</v>
+          <t>Casa amoblada para 7 personas con garaje</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>90714</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Estado: DENTRO</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="n">
-        <v>289850</v>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>2028950</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Puntaje</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>74.8</v>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Casa para 8 personas</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>124151</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Casa con piscina privada</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Sí (anuncio)</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>430608</v>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Enlace</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>https://www.hostelworld.com/hostels/p/329092/la-chanca-hostel/</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>No cumplen (por qué se miran baños y camas, no solo el precio):</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Casa Familiar 5 Hab con Terraza — San Antonio, $77.042 pp · 6 camas · 1 baños → La más barata del barrido, pero 1 solo baño para 11 personas → justo lo que no queremos.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
-        <is>
-          <t>Calificación huéspedes</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="n">
-        <v>9.800000000000001</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>Aire acondicionado</t>
-        </is>
-      </c>
-      <c r="B13" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>Piscina</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>Zona</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="inlineStr">
-        <is>
-          <t>San Antonio</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Apto El Ingenio 301 — El Ingenio (sur), $147.857 pp · 3 camas · 2 baños → Solo 3 camas (bajo el mínimo de 5) y lejos de la rumba de San Antonio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A11:I11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2089,14 +2411,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Amenidades en meta</t>
+          <t>Económico</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Piscina y aire acondicionado sin salir de los 400 mil. La alternativa prudente de presupuesto.</t>
+          <t>Máximo ahorro y el mejor rating del barrido (9.8). San Antonio, amenidades básicas.</t>
         </is>
       </c>
     </row>
@@ -2130,14 +2452,14 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Hostal Patio del Río</t>
+          <t>La Chanca Hostel</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>189750</v>
+        <v>89850</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1328250</v>
+        <v>628950</v>
       </c>
     </row>
     <row r="6">
@@ -2170,10 +2492,10 @@
         </is>
       </c>
       <c r="C7" s="22" t="n">
-        <v>389750</v>
+        <v>289850</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>2728250</v>
+        <v>2028950</v>
       </c>
     </row>
     <row r="9">
@@ -2183,7 +2505,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>72.8</v>
+        <v>74.8</v>
       </c>
     </row>
     <row r="10">
@@ -2194,7 +2516,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>https://www.hostelworld.com/hostels/p/323610/hostal-patio-del-rio/</t>
+          <t>https://www.hostelworld.com/hostels/p/329092/la-chanca-hostel/</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2527,7 @@
         </is>
       </c>
       <c r="B12" s="23" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2216,7 +2538,7 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2550,7 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2562,7 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2574,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Oeste (Cali)</t>
+          <t>San Antonio</t>
         </is>
       </c>
     </row>
@@ -2286,14 +2608,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>El equilibrio</t>
+          <t>Amenidades en meta</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Seguridad, piscina, aire, bar, rumba a pie y ambiente social. El puntaje más alto.</t>
+          <t>Piscina y aire acondicionado sin salir de los 400 mil. La alternativa prudente de presupuesto.</t>
         </is>
       </c>
     </row>
@@ -2327,14 +2649,14 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Viajero Hostel &amp; Salsa School</t>
+          <t>Hostal Patio del Río</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>252282</v>
+        <v>189750</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1765974</v>
+        <v>1328250</v>
       </c>
     </row>
     <row r="6">
@@ -2356,21 +2678,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Estado: FLEX</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>452282</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>3165974</v>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Estado: DENTRO</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>389750</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>2728250</v>
       </c>
     </row>
     <row r="9">
@@ -2380,7 +2702,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>72.8</v>
       </c>
     </row>
     <row r="10">
@@ -2391,7 +2713,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>https://www.hostelworld.com/hostels/p/73676/viajero-cali-hostel-and-salsa-school/</t>
+          <t>https://www.hostelworld.com/hostels/p/323610/hostal-patio-del-rio/</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2771,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Oeste (Cali)</t>
         </is>
       </c>
     </row>
@@ -2483,14 +2805,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Casa entera</t>
+          <t>El equilibrio</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Máxima privacidad y comodidad (piscina, aire, cocina). Dentro del flex.</t>
+          <t>Seguridad, piscina, aire, bar, rumba a pie y ambiente social. El puntaje más alto.</t>
         </is>
       </c>
     </row>
@@ -2524,14 +2846,14 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Casa/Apto entero (Airbnb)</t>
+          <t>Viajero Hostel &amp; Salsa School</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>300000</v>
+        <v>252282</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2100000</v>
+        <v>1765974</v>
       </c>
     </row>
     <row r="6">
@@ -2553,21 +2875,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Estado: EXCEDE</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="n">
-        <v>500000</v>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>3500000</v>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Estado: FLEX</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>452282</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>3165974</v>
       </c>
     </row>
     <row r="9">
@@ -2577,7 +2899,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>71.2</v>
+        <v>77.59999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -2588,7 +2910,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>https://www.airbnb.com/s/San-Antonio--Cali--Valle-del-Cauca/homes?checkin=2026-10-30&amp;checkout=2026-11-02&amp;adults=7</t>
+          <t>https://www.hostelworld.com/hostels/p/73676/viajero-cali-hostel-and-salsa-school/</t>
         </is>
       </c>
     </row>
@@ -2598,10 +2920,8 @@
           <t>Calificación huéspedes</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B12" s="23" t="n">
+        <v>9.6</v>
       </c>
     </row>
     <row r="13">
@@ -2636,7 +2956,7 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2968,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>San Antonio (Oeste)</t>
+          <t>San Antonio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Airbnb v5: saca Casa 7p (fea) y Refugio (dispo/cara), suma 2 del noroeste; ★ = mejor con cama
- El usuario descartó Casa 7p garaje (poco atractiva) y Refugio Vistas (noches no disponibles
  + cara). Van a descartes con su razón.
- Promovidas las dos mejores del noroeste que quedaban: Apto Granada/Chipichape (~1,8 km, la
  más céntrica y barata) y Torre Gardes (~3 km, piscina, 4 baños, 5.0). Set de 4.
- La ★ ya no es la de mayor puntaje sino la mejor CON cama para los 7 (camas>=5): La Flora
  (7 camas). La #1 por puntaje (Granada/Chipichape, 77.2) es más barata/céntrica pero 4 camas;
  se explica el matiz en informe/PDF/tarjeta del gráfico.
- Normalización de precio dentro del set, pero con 4 ítems (con 2 casi iguales se distorsionaba).
- Actualiza D-005 (v5).
</commit_message>
<xml_diff>
--- a/output/Mini-Boom-en-Cali_Resultados.xlsx
+++ b/output/Mini-Boom-en-Cali_Resultados.xlsx
@@ -2149,7 +2149,7 @@
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Alojamiento entero, 7 personas, noroeste/oeste cerca de actividades. Ubicación verificada por COORDENADAS ('Dist.' = km a Granada/El Peñón). Mismo puntaje 0–100 que los hostales, precio normalizado entre casas. Mejor: Agradable y Hermoso Apartamento (La Flora) (72.4/100). Disponibilidad del rango (30→2) y aire/piscina: confirmar al reservar.</t>
+          <t>Alojamiento entero, 7 personas, noroeste/oeste cerca de actividades. Ubicación verificada por COORDENADAS ('Dist.' = km a Granada/El Peñón). Mismo puntaje 0–100 que los hostales, precio normalizado entre casas. Mejor: Agradable y Hermoso Apartamento (La Flora) (74.6/100). Disponibilidad del rango (30→2) y aire/piscina: confirmar al reservar.</t>
         </is>
       </c>
     </row>
@@ -2206,78 +2206,78 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Apto Granada / Chipichape (fresco)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>129771</v>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Agradable y Hermoso Apartamento (La Flora) ★</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Norte (La Flora)</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C6" s="15" t="n">
         <v>4.8</v>
       </c>
-      <c r="D5" s="18" t="n">
-        <v>72.40000000000001</v>
-      </c>
-      <c r="E5" s="15" t="n">
+      <c r="D6" s="18" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="E6" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F6" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H6" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I6" s="13" t="n">
         <v>185894</v>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Casa amoblada para 7 personas con garaje</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Centro-oeste</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="D6" s="19" t="n">
-        <v>70.8</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>4.97</v>
-      </c>
-      <c r="I6" s="10" t="n">
-        <v>90714</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v>0.6</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>65.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>6</v>
@@ -2328,36 +2328,36 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Espacioso refugio de 3 dormitorios – Vistas</t>
+          <t>Torre Gardes</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Oeste (ladera)</t>
+          <t>Noroeste</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>63.2</v>
+        <v>66.8</v>
       </c>
       <c r="E8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>4.84</v>
-      </c>
       <c r="I8" s="10" t="n">
-        <v>282068</v>
+        <v>285714</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
@@ -2375,14 +2375,14 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Apto Granada / Chipichape (fresco) — Noroeste ~1,8 km, $129.771 pp · 4 camas · 2.5 baños → Muy bien ubicado (noroeste, ~1,8 km) y 2,5 baños, pero solo 4 camas (&lt;5 para los siete).</t>
+          <t>Casa amoblada para 7 personas con garaje — Centro-oeste ~3,6 km, $90.714 pp · 5 camas · 2.5 baños → La descartaste: poco atractiva, aunque era barata (5 camas, garaje).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Torre Gardes — Noroeste ~3,0 km, $285.714 pp · 4 camas · 4 baños → Noroeste, piscina, 4 baños y rating 5,0 — pero 4 camas (&lt;5) y caro.</t>
+          <t>Espacioso refugio de 3 dormitorios – Vistas — Oeste ~2,4 km, $282.068 pp · 5 camas · 3 baños → La descartaste: las noches no cuadran y es cara (~$282k pp).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Airbnb v7: integra las 4 opciones del usuario al cuadro, TODAS medidas, marcadas por tipo
'márcalas donde van' = medirlas con el algoritmo, no excluirlas. El cuadro de Airbnb ahora
incluye las 6 (las 4 del usuario + 2 casas enteras verificadas), todas puntuadas, con columnas
nuevas Tipo (entero/apartahotel/hotel/hab. compartida) y ¿Baño comp.?:
  1. La Flora (Entero, 80.1) ★   2. Lofthouse (Apartahotel, 77.9)   3. Hotel (77.9)
  4. Hab. compartida (75.0, baño Sí-extraños)   5. Casa-museo (73.2)   6. Apto servicios (66.8)
- La ★ se restringe a la mejor CASA ENTERA con camas>=5 (no un hotel).
- camas/banos/rating pueden ser None (hoteles) -> '—' (helper dash()).
- Descartes solo para las que NO tienen el rango 30->2. Columna Total (3n) + por persona en los 4.
Actualiza D-005 (v7).
</commit_message>
<xml_diff>
--- a/output/Mini-Boom-en-Cali_Resultados.xlsx
+++ b/output/Mini-Boom-en-Cali_Resultados.xlsx
@@ -2127,13 +2127,13 @@
   <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -2143,51 +2143,51 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🛏️ Airbnb — casas/aptos ENTEROS en el noroeste/oeste (disponibilidad 30→2 verificada)</t>
+          <t>🛏️ Airbnb — alojamientos considerados (noroeste/oeste, disponibilidad 30→2 verificada)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Solo alojamientos enteros (ningún baño compartido), 7 personas. Ubicación por COORDENADAS ('Dist.' = km a Granada/El Peñón) y rango 30→2 verificado en el calendario real. Mismo puntaje 0–100 que los hostales. Mejor con cama para los 7: Vivienda entera (La Flora) (80.1/100). Aire: confirmar al reservar.</t>
+          <t>Todas las opciones puestas sobre la mesa, 7 personas, marcadas por TIPO (entero/apartahotel/hotel/hab. compartida) y si el baño se comparte. Rango 30→2 verificado en el calendario real; ubicación por coordenadas. Mismo puntaje 0–100 que los hostales. Mejor casa entera para los 7: Vivienda entera (La Flora) (80.1/100). Camas/baños «—» = por unidad.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Casa / apto entero</t>
+          <t>Alojamiento</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>¿Baño comp.?</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
           <t>Dist. (km)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Puntaje</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Camas</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Baños</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Aire</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -2219,28 +2219,34 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Norte (La Flora)</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="n">
+          <t>Entero</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="n">
         <v>4.8</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="E5" s="18" t="n">
         <v>80.09999999999999</v>
       </c>
-      <c r="E5" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="F5" s="15" t="n">
-        <v>2</v>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H5" s="15" t="n">
-        <v>5</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
       </c>
       <c r="I5" s="13" t="n">
         <v>1301262</v>
@@ -2257,39 +2263,45 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Casa-museo Fundación Cerón (San Antonio)</t>
+          <t>Lofthouse 14 (apartahotel)</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Oeste (San Antonio)</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D6" s="19" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>2.5</v>
+          <t>Apartahotel</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>No (unidad)</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="11" t="n">
-        <v>4.63</v>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>4.92</t>
+        </is>
       </c>
       <c r="I6" s="10" t="n">
-        <v>1294200</v>
+        <v>1489745</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>184885</v>
+        <v>212820</v>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
@@ -2300,71 +2312,203 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Apartamento entero con servicios (tu hallazgo)</t>
+          <t>Habitación en hotel</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Oeste</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>No (unidad)</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>1489745</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>212820</v>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Habitación compartida (casa de huéspedes)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Hab. compartida</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Sí (extraños)</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>75</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>4.67</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>1440622</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>205803</v>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Casa-museo Fundación Cerón (San Antonio)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Entero</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>2,5</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>4.63</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>1294200</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>184885</v>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Apartamento entero con servicios</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Entero</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n">
         <v>3.6</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="E10" s="19" t="n">
         <v>66.8</v>
       </c>
-      <c r="E7" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>4.87</v>
-      </c>
-      <c r="I7" s="6" t="n">
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>4.87</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="n">
         <v>1723404</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J10" s="10" t="n">
         <v>246200</v>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Marcadas donde van — no son casa entera o no tienen el rango 30→2 (verificado):</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Hab. compartida en casa de huéspedes — Oeste ~3,1 km, total $1.440.622 → $205.803 pp · 9 camas · 6 baños → Es una HABITACIÓN COMPARTIDA con 6 baños COMPARTIDOS → va contra lo de no compartir baño con extraños.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Lofthouse 14 (apartahotel) — Oeste ~2,0 km, total $1.489.745 → $212.820 pp → Es un APARTAHOTEL (habitación en hotel), no una casa entera. Privado y con aire, pero formato hotel.</t>
-        </is>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Habitación en hotel — Oeste ~2,1 km, total $1.489.745 → $212.820 pp → Es un HOTEL (habitación), no una casa entera.</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Fuera por disponibilidad — el calendario NO tiene el rango 30→2 (verificado):</t>
         </is>
       </c>
     </row>
@@ -2383,20 +2527,19 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A12:K12"/>
+  <mergeCells count="4">
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A11:K11"/>
-    <mergeCell ref="A10:K10"/>
-    <mergeCell ref="A13:K13"/>
     <mergeCell ref="A14:K14"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A13:K13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>